<commit_message>
updated documentation, usecase diagrams, and budget
</commit_message>
<xml_diff>
--- a/Budget.xlsx
+++ b/Budget.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stevens0-my.sharepoint.com/personal/rdavis2_stevens_edu/Documents/senior_year/ssw423-senior_design/findIt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{B70044C6-B3F8-2B40-A8E0-66A11601ED6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3213A8EC-3D72-DD49-9654-6024315BC708}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{B70044C6-B3F8-2B40-A8E0-66A11601ED6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DBBD3FC-B47E-4EE4-BC05-749C5D609C71}"/>
   <bookViews>
     <workbookView xWindow="940" yWindow="500" windowWidth="27480" windowHeight="16940" xr2:uid="{AD84C507-867E-B745-ABC7-19A34880FDF6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Item</t>
   </si>
@@ -54,6 +54,12 @@
   </si>
   <si>
     <t>Wio Tracker 1110 Digikey</t>
+  </si>
+  <si>
+    <t>Sum:</t>
+  </si>
+  <si>
+    <t>Remaining Budget</t>
   </si>
 </sst>
 </file>
@@ -107,7 +113,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
@@ -457,10 +463,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{742BA98A-704C-5D41-BE1D-D0E7A2333F77}">
-  <dimension ref="B2:E3"/>
+  <dimension ref="B2:E17"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
-    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -490,6 +496,24 @@
       </c>
       <c r="E3">
         <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5">
+      <c r="C16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="2">
+        <f>SUM(D3:D15)</f>
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4">
+      <c r="C17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="2">
+        <f>700-D16</f>
+        <v>670.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>